<commit_message>
Add Week 6 booked hours
</commit_message>
<xml_diff>
--- a/Documentation/Week 5/Booked Hours/Booked_Hours_Murphy.xlsx
+++ b/Documentation/Week 5/Booked Hours/Booked_Hours_Murphy.xlsx
@@ -1,41 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr date1904="1"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24314441_student_uwa_edu_au/Documents/UWA/Year 3/Sem 2/CITS3200_Project/Documentation/Week 5/Booked Hours/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_D968DDC6C1ECB36C98BB40744087C10C33359316" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="24200" windowHeight="11980" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="BookedHours" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="21">
   <si>
     <r>
       <rPr>
@@ -112,16 +93,26 @@
   <si>
     <t>Adjust the github, merge branches</t>
   </si>
+  <si>
+    <t>First Audit Meeting</t>
+  </si>
+  <si>
+    <t>First Mentor Meeting</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="168" formatCode="dd/mm/yy"/>
-    <numFmt numFmtId="169" formatCode="h:mm;@"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="6">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="dd/mm/yy"/>
+    <numFmt numFmtId="177" formatCode="h:mm;@"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="24">
     <font>
       <sz val="10"/>
       <name val="Verdana"/>
@@ -140,20 +131,357 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
       <name val="Lucida Sans"/>
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -301,15 +629,281 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="13" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
@@ -318,11 +912,11 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -334,63 +928,90 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  <cellStyles count="49">
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <colors>
     <indexedColors>
@@ -463,9 +1084,6 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -787,297 +1405,297 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:I132"/>
-  <sheetFormatPr defaultColWidth="10.6328125" defaultRowHeight="12.6"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.2"/>
   <cols>
-    <col min="1" max="1" width="5.81640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.90625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.1796875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.36328125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.36328125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="69.26953125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9.36328125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="12.7265625" style="1"/>
-    <col min="9" max="9" width="10.6328125" style="1" hidden="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.6328125" style="1"/>
+    <col min="1" max="1" width="5.8359375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.9296875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.1640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.3359375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.359375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="69.2578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="9.3359375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6875" style="1"/>
+    <col min="9" max="9" width="10.6640625" style="1" hidden="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="70.95" customHeight="1">
-      <c r="A1" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="11"/>
-    </row>
-    <row r="2" spans="1:9" ht="16.05" customHeight="1">
-      <c r="A2" s="14" t="s">
+    <row r="1" ht="71" customHeight="1" spans="1:8">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="14"/>
+    </row>
+    <row r="2" ht="16" customHeight="1" spans="1:8">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="12" t="s">
+      <c r="C2" s="6"/>
+      <c r="D2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="13"/>
-      <c r="F2" s="16" t="s">
+      <c r="E2" s="6"/>
+      <c r="F2" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="16" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="13.05" customHeight="1">
-      <c r="A3" s="15"/>
-      <c r="B3" s="2" t="s">
+    <row r="3" ht="13" customHeight="1" spans="1:8">
+      <c r="A3" s="7"/>
+      <c r="B3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="9" t="s">
         <v>8</v>
       </c>
       <c r="F3" s="17"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="20"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="18"/>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="10">
         <v>44770</v>
       </c>
-      <c r="C4" s="5">
-        <v>0.45833333333333298</v>
-      </c>
-      <c r="D4" s="4">
+      <c r="C4" s="11">
+        <v>0.458333333333333</v>
+      </c>
+      <c r="D4" s="10">
         <v>44770</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="11">
         <v>0.5</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="19">
         <f t="shared" ref="G4:G16" si="0">IF(I4&gt;0,I4,IF(I4=0," ","ERROR"))</f>
-        <v>0.99999999994179234</v>
+        <v>0.999999999941792</v>
       </c>
       <c r="H4" s="1">
         <f>IF(G4&lt;&gt;"ERROR",G4)</f>
-        <v>0.99999999994179234</v>
+        <v>0.999999999941792</v>
       </c>
       <c r="I4" s="1">
         <f t="shared" ref="I4:I16" si="1">((D4+E4)-(B4+C4))*24</f>
-        <v>0.99999999994179234</v>
+        <v>0.999999999941792</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="1">
         <v>2</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="10">
         <v>44771</v>
       </c>
-      <c r="C5" s="5">
-        <v>0.64583333333333304</v>
-      </c>
-      <c r="D5" s="4">
+      <c r="C5" s="11">
+        <v>0.645833333333333</v>
+      </c>
+      <c r="D5" s="10">
         <v>44771</v>
       </c>
-      <c r="E5" s="5">
-        <v>0.72916666666666696</v>
+      <c r="E5" s="11">
+        <v>0.729166666666667</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="19">
         <f t="shared" si="0"/>
-        <v>1.9999999998835847</v>
+        <v>1.99999999988358</v>
       </c>
       <c r="H5" s="1">
         <f t="shared" ref="H5:H17" si="2">IF(AND(G5&lt;&gt;" ",G5&lt;&gt;"ERROR",H4&lt;&gt;" ",H4&lt;&gt;"ERROR"),G5+H4," ")</f>
-        <v>2.999999999825377</v>
+        <v>2.99999999982538</v>
       </c>
       <c r="I5" s="1">
         <f t="shared" si="1"/>
-        <v>1.9999999998835847</v>
+        <v>1.99999999988358</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="1">
         <v>3</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="10">
         <v>44777</v>
       </c>
-      <c r="C6" s="6">
-        <v>0.45833333333333298</v>
-      </c>
-      <c r="D6" s="4">
+      <c r="C6" s="12">
+        <v>0.458333333333333</v>
+      </c>
+      <c r="D6" s="10">
         <v>44777</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="12">
         <v>0.5</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="19">
         <f t="shared" si="0"/>
-        <v>0.99999999994179234</v>
+        <v>0.999999999941792</v>
       </c>
       <c r="H6" s="1">
         <f t="shared" si="2"/>
-        <v>3.9999999997671694</v>
+        <v>3.99999999976717</v>
       </c>
       <c r="I6" s="1">
         <f t="shared" si="1"/>
-        <v>0.99999999994179234</v>
+        <v>0.999999999941792</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="1">
         <v>3</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="10">
         <v>44777</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="12">
         <v>0.5</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="10">
         <v>44777</v>
       </c>
-      <c r="E7" s="6">
-        <v>0.54166666666666696</v>
+      <c r="E7" s="12">
+        <v>0.541666666666667</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="19">
         <f t="shared" si="0"/>
-        <v>0.99999999994179234</v>
+        <v>0.999999999941792</v>
       </c>
       <c r="H7" s="1">
         <f t="shared" si="2"/>
-        <v>4.9999999997089617</v>
+        <v>4.99999999970896</v>
       </c>
       <c r="I7" s="1">
         <f t="shared" si="1"/>
-        <v>0.99999999994179234</v>
+        <v>0.999999999941792</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="1">
         <v>3</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="10">
         <v>44777</v>
       </c>
-      <c r="C8" s="6">
-        <v>0.54166666666666696</v>
-      </c>
-      <c r="D8" s="4">
+      <c r="C8" s="12">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="D8" s="10">
         <v>44777</v>
       </c>
-      <c r="E8" s="6">
-        <v>0.58333333333333304</v>
+      <c r="E8" s="12">
+        <v>0.583333333333333</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="19">
         <f t="shared" si="0"/>
-        <v>1.0000000001164153</v>
+        <v>1.00000000011642</v>
       </c>
       <c r="H8" s="1">
         <f t="shared" si="2"/>
-        <v>5.999999999825377</v>
+        <v>5.99999999982538</v>
       </c>
       <c r="I8" s="1">
         <f t="shared" si="1"/>
-        <v>1.0000000001164153</v>
+        <v>1.00000000011642</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="1">
         <v>3</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="10">
         <v>44777</v>
       </c>
-      <c r="C9" s="6">
-        <v>0.58333333333333304</v>
-      </c>
-      <c r="D9" s="4">
+      <c r="C9" s="12">
+        <v>0.583333333333333</v>
+      </c>
+      <c r="D9" s="10">
         <v>44777</v>
       </c>
-      <c r="E9" s="6">
-        <v>0.66666666666666696</v>
+      <c r="E9" s="12">
+        <v>0.666666666666667</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="19">
         <f t="shared" si="0"/>
-        <v>1.9999999998835847</v>
+        <v>1.99999999988358</v>
       </c>
       <c r="H9" s="1">
         <f t="shared" si="2"/>
-        <v>7.9999999997089617</v>
+        <v>7.99999999970896</v>
       </c>
       <c r="I9" s="1">
         <f t="shared" si="1"/>
-        <v>1.9999999998835847</v>
+        <v>1.99999999988358</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="1">
         <v>3</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="10">
         <v>44779</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="12">
         <v>0.625</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="10">
         <v>44779</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="12">
         <v>0.6875</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="19">
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
       <c r="H10" s="1">
         <f t="shared" si="2"/>
-        <v>9.4999999997089617</v>
+        <v>9.49999999970896</v>
       </c>
       <c r="I10" s="1">
         <f t="shared" si="1"/>
@@ -1088,124 +1706,124 @@
       <c r="A11" s="1">
         <v>4</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="10">
         <v>44783</v>
       </c>
-      <c r="C11" s="6">
-        <v>0.66666666666666696</v>
-      </c>
-      <c r="D11" s="4">
+      <c r="C11" s="12">
+        <v>0.666666666666667</v>
+      </c>
+      <c r="D11" s="10">
         <v>44783</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="12">
         <v>0.75</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="8">
+      <c r="G11" s="19">
         <f t="shared" si="0"/>
-        <v>2.0000000000582077</v>
+        <v>2.00000000005821</v>
       </c>
       <c r="H11" s="1">
         <f t="shared" si="2"/>
-        <v>11.499999999767169</v>
+        <v>11.4999999997672</v>
       </c>
       <c r="I11" s="1">
         <f t="shared" si="1"/>
-        <v>2.0000000000582077</v>
+        <v>2.00000000005821</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="1">
         <v>4</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="10">
         <v>44784</v>
       </c>
-      <c r="C12" s="6">
-        <v>0.45833333333333298</v>
-      </c>
-      <c r="D12" s="4">
+      <c r="C12" s="12">
+        <v>0.458333333333333</v>
+      </c>
+      <c r="D12" s="10">
         <v>44784</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="12">
         <v>0.5</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G12" s="8">
+      <c r="G12" s="19">
         <f t="shared" si="0"/>
-        <v>0.99999999994179234</v>
+        <v>0.999999999941792</v>
       </c>
       <c r="H12" s="1">
         <f t="shared" si="2"/>
-        <v>12.499999999708962</v>
+        <v>12.499999999709</v>
       </c>
       <c r="I12" s="1">
         <f t="shared" si="1"/>
-        <v>0.99999999994179234</v>
+        <v>0.999999999941792</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="1">
         <v>4</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="10">
         <v>44784</v>
       </c>
-      <c r="C13" s="6">
-        <v>0.54166666666666696</v>
-      </c>
-      <c r="D13" s="4">
+      <c r="C13" s="12">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="D13" s="10">
         <v>44784</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="12">
         <v>0.5625</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="19">
         <f t="shared" si="0"/>
-        <v>0.50000000005820766</v>
+        <v>0.500000000058208</v>
       </c>
       <c r="H13" s="1">
         <f t="shared" si="2"/>
-        <v>12.999999999767169</v>
+        <v>12.9999999997672</v>
       </c>
       <c r="I13" s="1">
         <f t="shared" si="1"/>
-        <v>0.50000000005820766</v>
+        <v>0.500000000058208</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="1">
         <v>4</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="10">
         <v>44786</v>
       </c>
-      <c r="C14" s="6">
-        <v>0.54166666666666696</v>
-      </c>
-      <c r="D14" s="4">
+      <c r="C14" s="12">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="D14" s="10">
         <v>44786</v>
       </c>
-      <c r="E14" s="6">
-        <v>0.60416666666666696</v>
+      <c r="E14" s="12">
+        <v>0.604166666666667</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="19">
         <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
       <c r="H14" s="1">
         <f t="shared" si="2"/>
-        <v>14.499999999767169</v>
+        <v>14.4999999997672</v>
       </c>
       <c r="I14" s="1">
         <f t="shared" si="1"/>
@@ -1216,393 +1834,435 @@
       <c r="A15" s="1">
         <v>4</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="10">
         <v>44787</v>
       </c>
-      <c r="C15" s="6">
-        <v>0.54166666666666696</v>
-      </c>
-      <c r="D15" s="4">
+      <c r="C15" s="12">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="D15" s="10">
         <v>44787</v>
       </c>
-      <c r="E15" s="6">
-        <v>0.64305555555555605</v>
+      <c r="E15" s="12">
+        <v>0.643055555555556</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="19">
         <f t="shared" si="0"/>
-        <v>2.433333333407063</v>
+        <v>2.43333333340706</v>
       </c>
       <c r="H15" s="1">
         <f t="shared" si="2"/>
-        <v>16.933333333174232</v>
+        <v>16.9333333331742</v>
       </c>
       <c r="I15" s="1">
         <f t="shared" si="1"/>
-        <v>2.433333333407063</v>
+        <v>2.43333333340706</v>
       </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="1">
         <v>5</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="10">
         <v>44789</v>
       </c>
-      <c r="C16" s="6">
-        <v>0.41666666666666702</v>
-      </c>
-      <c r="D16" s="4">
+      <c r="C16" s="12">
+        <v>0.416666666666667</v>
+      </c>
+      <c r="D16" s="10">
         <v>44789</v>
       </c>
-      <c r="E16" s="6">
-        <v>0.57222222222222197</v>
+      <c r="E16" s="12">
+        <v>0.572222222222222</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="19">
         <f t="shared" si="0"/>
-        <v>3.7333333334536292</v>
+        <v>3.73333333345363</v>
       </c>
       <c r="H16" s="1">
         <f t="shared" si="2"/>
-        <v>20.666666666627862</v>
+        <v>20.6666666666279</v>
       </c>
       <c r="I16" s="1">
         <f t="shared" si="1"/>
-        <v>3.7333333334536292</v>
+        <v>3.73333333345363</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="1">
         <v>5</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="10">
         <v>44789</v>
       </c>
-      <c r="C17" s="6">
+      <c r="C17" s="12">
         <v>0.625</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="10">
         <v>44789</v>
       </c>
-      <c r="E17" s="6">
-        <v>0.66666666666666696</v>
+      <c r="E17" s="12">
+        <v>0.666666666666667</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="19">
         <f t="shared" ref="G17:G30" si="3">IF(I17&gt;0,I17,IF(I17=0," ","ERROR"))</f>
-        <v>0.99999999994179234</v>
+        <v>0.999999999941792</v>
       </c>
       <c r="H17" s="1">
         <f t="shared" si="2"/>
-        <v>21.666666666569654</v>
+        <v>21.6666666665697</v>
       </c>
       <c r="I17" s="1">
         <f t="shared" ref="I17:I68" si="4">((D17+E17)-(B17+C17))*24</f>
-        <v>0.99999999994179234</v>
+        <v>0.999999999941792</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="1">
         <v>5</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="10">
         <v>44791</v>
       </c>
-      <c r="C18" s="6">
-        <v>0.45833333333333298</v>
-      </c>
-      <c r="D18" s="4">
+      <c r="C18" s="12">
+        <v>0.458333333333333</v>
+      </c>
+      <c r="D18" s="10">
         <v>44791</v>
       </c>
-      <c r="E18" s="6">
-        <v>0.52638888888888902</v>
+      <c r="E18" s="12">
+        <v>0.526388888888889</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="G18" s="8">
+      <c r="G18" s="19">
         <f t="shared" si="3"/>
-        <v>1.6333333332440816</v>
+        <v>1.63333333324408</v>
       </c>
       <c r="H18" s="1">
-        <f t="shared" ref="H18:H30" si="5">IF(AND(G18&lt;&gt;" ",G18&lt;&gt;"ERROR",H17&lt;&gt;" ",H17&lt;&gt;"ERROR"),G18+H17," ")</f>
-        <v>23.299999999813735</v>
+        <f t="shared" ref="H17:H30" si="5">IF(AND(G18&lt;&gt;" ",G18&lt;&gt;"ERROR",H17&lt;&gt;" ",H17&lt;&gt;"ERROR"),G18+H17," ")</f>
+        <v>23.2999999998138</v>
       </c>
       <c r="I18" s="1">
         <f t="shared" si="4"/>
-        <v>1.6333333332440816</v>
+        <v>1.63333333324408</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" s="1">
         <v>5</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="10">
         <v>44791</v>
       </c>
-      <c r="C19" s="6">
-        <v>0.54166666666666696</v>
-      </c>
-      <c r="D19" s="4">
+      <c r="C19" s="12">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="D19" s="10">
         <v>44791</v>
       </c>
-      <c r="E19" s="6">
-        <v>0.58333333333333304</v>
+      <c r="E19" s="12">
+        <v>0.583333333333333</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G19" s="8">
+      <c r="G19" s="19">
         <f t="shared" si="3"/>
-        <v>1.0000000001164153</v>
+        <v>1.00000000011642</v>
       </c>
       <c r="H19" s="1">
         <f t="shared" si="5"/>
-        <v>24.299999999930151</v>
+        <v>24.2999999999302</v>
       </c>
       <c r="I19" s="1">
         <f t="shared" si="4"/>
-        <v>1.0000000001164153</v>
+        <v>1.00000000011642</v>
       </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="1">
         <v>5</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="10">
         <v>44793</v>
       </c>
-      <c r="C20" s="6">
-        <v>0.85416666666666696</v>
-      </c>
-      <c r="D20" s="4">
+      <c r="C20" s="12">
+        <v>0.854166666666667</v>
+      </c>
+      <c r="D20" s="10">
         <v>44793</v>
       </c>
-      <c r="E20" s="6">
+      <c r="E20" s="12">
         <v>0.875</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G20" s="8">
+      <c r="G20" s="19">
         <f t="shared" si="3"/>
-        <v>0.50000000005820766</v>
+        <v>0.500000000058208</v>
       </c>
       <c r="H20" s="1">
         <f t="shared" si="5"/>
-        <v>24.799999999988358</v>
+        <v>24.7999999999884</v>
       </c>
       <c r="I20" s="1">
         <f t="shared" si="4"/>
-        <v>0.50000000005820766</v>
+        <v>0.500000000058208</v>
       </c>
     </row>
     <row r="21" spans="1:9">
-      <c r="B21" s="7"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="6"/>
-      <c r="G21" s="8" t="str">
+      <c r="A21" s="1">
+        <v>6</v>
+      </c>
+      <c r="B21" s="10">
+        <v>44798</v>
+      </c>
+      <c r="C21" s="12">
+        <v>0.458333333333333</v>
+      </c>
+      <c r="D21" s="10">
+        <v>44798</v>
+      </c>
+      <c r="E21" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G21" s="19">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H21" s="1" t="str">
+        <v>0.999999999941792</v>
+      </c>
+      <c r="H21" s="1">
         <f t="shared" si="5"/>
-        <v xml:space="preserve"> </v>
+        <v>25.7999999999302</v>
       </c>
       <c r="I21" s="1">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.999999999941792</v>
       </c>
     </row>
     <row r="22" spans="1:9">
-      <c r="B22" s="7"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="6"/>
-      <c r="G22" s="8" t="str">
+      <c r="A22" s="1">
+        <v>6</v>
+      </c>
+      <c r="B22" s="10">
+        <v>44798</v>
+      </c>
+      <c r="C22" s="12">
+        <v>0.5</v>
+      </c>
+      <c r="D22" s="10">
+        <v>44798</v>
+      </c>
+      <c r="E22" s="20">
+        <v>0.541666666666667</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G22" s="19">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H22" s="1" t="str">
+        <v>0.999999999941792</v>
+      </c>
+      <c r="H22" s="1">
         <f t="shared" si="5"/>
-        <v xml:space="preserve"> </v>
+        <v>26.799999999872</v>
       </c>
       <c r="I22" s="1">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.999999999941792</v>
       </c>
     </row>
     <row r="23" spans="1:9">
-      <c r="B23" s="7"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="6"/>
-      <c r="G23" s="8" t="str">
+      <c r="A23" s="1">
+        <v>6</v>
+      </c>
+      <c r="B23" s="10">
+        <v>44800</v>
+      </c>
+      <c r="C23" s="12">
+        <v>0.652777777777778</v>
+      </c>
+      <c r="D23" s="10">
+        <v>44800</v>
+      </c>
+      <c r="E23" s="12">
+        <v>0.666666666666667</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G23" s="19">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H23" s="1" t="str">
+        <v>0.333333333197515</v>
+      </c>
+      <c r="H23" s="1">
         <f t="shared" si="5"/>
-        <v xml:space="preserve"> </v>
+        <v>27.1333333330695</v>
       </c>
       <c r="I23" s="1">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="B24" s="7"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="6"/>
-      <c r="G24" s="8" t="str">
+        <v>0.333333333197515</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9">
+      <c r="B24" s="13"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="12"/>
+      <c r="G24" s="19" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H24" s="1" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I24" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
-      <c r="B25" s="7"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="6"/>
-      <c r="G25" s="8" t="str">
+    <row r="25" spans="2:9">
+      <c r="B25" s="13"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="12"/>
+      <c r="G25" s="19" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H25" s="1" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I25" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
-      <c r="B26" s="7"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="6"/>
-      <c r="G26" s="8" t="str">
+    <row r="26" spans="2:9">
+      <c r="B26" s="13"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="12"/>
+      <c r="G26" s="19" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H26" s="1" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I26" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
-      <c r="B27" s="7"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="6"/>
-      <c r="G27" s="8" t="str">
+    <row r="27" spans="2:9">
+      <c r="B27" s="13"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="12"/>
+      <c r="G27" s="19" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H27" s="1" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I27" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
-      <c r="B28" s="7"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="6"/>
-      <c r="G28" s="8" t="str">
+    <row r="28" spans="2:9">
+      <c r="B28" s="13"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="12"/>
+      <c r="G28" s="19" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H28" s="1" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I28" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
-      <c r="B29" s="7"/>
-      <c r="C29" s="6"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="6"/>
-      <c r="G29" s="8" t="str">
+    <row r="29" spans="2:9">
+      <c r="B29" s="13"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="12"/>
+      <c r="G29" s="19" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H29" s="1" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I29" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
-      <c r="B30" s="7"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="6"/>
-      <c r="G30" s="8" t="str">
+    <row r="30" spans="2:9">
+      <c r="B30" s="13"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="12"/>
+      <c r="G30" s="19" t="str">
         <f t="shared" si="3"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H30" s="1" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I30" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="15">
-      <c r="A31" s="14" t="s">
+    <row r="31" ht="17.6" spans="1:9">
+      <c r="A31" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B31" s="12" t="s">
+      <c r="B31" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C31" s="13"/>
-      <c r="D31" s="12" t="s">
+      <c r="C31" s="6"/>
+      <c r="D31" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E31" s="13"/>
-      <c r="F31" s="18" t="s">
+      <c r="E31" s="6"/>
+      <c r="F31" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="G31" s="18" t="s">
+      <c r="G31" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="H31" s="18" t="s">
+      <c r="H31" s="21" t="s">
         <v>6</v>
       </c>
       <c r="I31" s="1" t="e">
@@ -1610,40 +2270,40 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="15">
-      <c r="A32" s="15"/>
-      <c r="B32" s="2" t="s">
+    <row r="32" ht="17.6" spans="1:9">
+      <c r="A32" s="7"/>
+      <c r="B32" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C32" s="3" t="s">
+      <c r="C32" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E32" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
       <c r="I32" s="1" t="e">
         <f t="shared" si="4"/>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="33" spans="2:9">
-      <c r="B33" s="7"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="6"/>
-      <c r="G33" s="8" t="str">
+      <c r="B33" s="13"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="12"/>
+      <c r="G33" s="19" t="str">
         <f t="shared" ref="G33:G64" si="6">IF(I33&gt;0,I33,IF(I33=0," ","ERROR"))</f>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H33" s="1" t="str">
         <f>IF(AND(G33&lt;&gt;" ",G33&lt;&gt;"ERROR",H30&lt;&gt;" ",H30&lt;&gt;"ERROR"),G33+H30," ")</f>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I33" s="1">
         <f t="shared" si="4"/>
@@ -1651,17 +2311,17 @@
       </c>
     </row>
     <row r="34" spans="2:9">
-      <c r="B34" s="7"/>
-      <c r="C34" s="6"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="6"/>
-      <c r="G34" s="8" t="str">
+      <c r="B34" s="13"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="12"/>
+      <c r="G34" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H34" s="1" t="str">
         <f t="shared" ref="H34:H64" si="7">IF(AND(G34&lt;&gt;" ",G34&lt;&gt;"ERROR",H33&lt;&gt;" ",H33&lt;&gt;"ERROR"),G34+H33," ")</f>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I34" s="1">
         <f t="shared" si="4"/>
@@ -1669,17 +2329,17 @@
       </c>
     </row>
     <row r="35" spans="2:9">
-      <c r="B35" s="7"/>
-      <c r="C35" s="6"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="6"/>
-      <c r="G35" s="8" t="str">
+      <c r="B35" s="13"/>
+      <c r="C35" s="12"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="12"/>
+      <c r="G35" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H35" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I35" s="1">
         <f t="shared" si="4"/>
@@ -1687,17 +2347,17 @@
       </c>
     </row>
     <row r="36" spans="2:9">
-      <c r="B36" s="7"/>
-      <c r="C36" s="6"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="6"/>
-      <c r="G36" s="8" t="str">
+      <c r="B36" s="13"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="12"/>
+      <c r="G36" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H36" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I36" s="1">
         <f t="shared" si="4"/>
@@ -1705,17 +2365,17 @@
       </c>
     </row>
     <row r="37" spans="2:9">
-      <c r="B37" s="7"/>
-      <c r="C37" s="6"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="6"/>
-      <c r="G37" s="8" t="str">
+      <c r="B37" s="13"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="12"/>
+      <c r="G37" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H37" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I37" s="1">
         <f t="shared" si="4"/>
@@ -1723,17 +2383,17 @@
       </c>
     </row>
     <row r="38" spans="2:9">
-      <c r="B38" s="7"/>
-      <c r="C38" s="6"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="6"/>
-      <c r="G38" s="8" t="str">
+      <c r="B38" s="13"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="12"/>
+      <c r="G38" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H38" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I38" s="1">
         <f t="shared" si="4"/>
@@ -1741,17 +2401,17 @@
       </c>
     </row>
     <row r="39" spans="2:9">
-      <c r="B39" s="7"/>
-      <c r="C39" s="6"/>
-      <c r="D39" s="7"/>
-      <c r="E39" s="6"/>
-      <c r="G39" s="8" t="str">
+      <c r="B39" s="13"/>
+      <c r="C39" s="12"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="12"/>
+      <c r="G39" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H39" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I39" s="1">
         <f t="shared" si="4"/>
@@ -1759,17 +2419,17 @@
       </c>
     </row>
     <row r="40" spans="2:9">
-      <c r="B40" s="7"/>
-      <c r="C40" s="6"/>
-      <c r="D40" s="7"/>
-      <c r="E40" s="6"/>
-      <c r="G40" s="8" t="str">
+      <c r="B40" s="13"/>
+      <c r="C40" s="12"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="12"/>
+      <c r="G40" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H40" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I40" s="1">
         <f t="shared" si="4"/>
@@ -1777,17 +2437,17 @@
       </c>
     </row>
     <row r="41" spans="2:9">
-      <c r="B41" s="7"/>
-      <c r="C41" s="6"/>
-      <c r="D41" s="7"/>
-      <c r="E41" s="6"/>
-      <c r="G41" s="8" t="str">
+      <c r="B41" s="13"/>
+      <c r="C41" s="12"/>
+      <c r="D41" s="13"/>
+      <c r="E41" s="12"/>
+      <c r="G41" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H41" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I41" s="1">
         <f t="shared" si="4"/>
@@ -1795,17 +2455,17 @@
       </c>
     </row>
     <row r="42" spans="2:9">
-      <c r="B42" s="7"/>
-      <c r="C42" s="6"/>
-      <c r="D42" s="7"/>
-      <c r="E42" s="6"/>
-      <c r="G42" s="8" t="str">
+      <c r="B42" s="13"/>
+      <c r="C42" s="12"/>
+      <c r="D42" s="13"/>
+      <c r="E42" s="12"/>
+      <c r="G42" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H42" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I42" s="1">
         <f t="shared" si="4"/>
@@ -1813,17 +2473,17 @@
       </c>
     </row>
     <row r="43" spans="2:9">
-      <c r="B43" s="7"/>
-      <c r="C43" s="6"/>
-      <c r="D43" s="7"/>
-      <c r="E43" s="6"/>
-      <c r="G43" s="8" t="str">
+      <c r="B43" s="13"/>
+      <c r="C43" s="12"/>
+      <c r="D43" s="13"/>
+      <c r="E43" s="12"/>
+      <c r="G43" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H43" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I43" s="1">
         <f t="shared" si="4"/>
@@ -1831,17 +2491,17 @@
       </c>
     </row>
     <row r="44" spans="2:9">
-      <c r="B44" s="7"/>
-      <c r="C44" s="6"/>
-      <c r="D44" s="7"/>
-      <c r="E44" s="6"/>
-      <c r="G44" s="8" t="str">
+      <c r="B44" s="13"/>
+      <c r="C44" s="12"/>
+      <c r="D44" s="13"/>
+      <c r="E44" s="12"/>
+      <c r="G44" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H44" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I44" s="1">
         <f t="shared" si="4"/>
@@ -1849,17 +2509,17 @@
       </c>
     </row>
     <row r="45" spans="2:9">
-      <c r="B45" s="7"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="7"/>
-      <c r="E45" s="6"/>
-      <c r="G45" s="8" t="str">
+      <c r="B45" s="13"/>
+      <c r="C45" s="12"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="12"/>
+      <c r="G45" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H45" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I45" s="1">
         <f t="shared" si="4"/>
@@ -1867,17 +2527,17 @@
       </c>
     </row>
     <row r="46" spans="2:9">
-      <c r="B46" s="7"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="7"/>
-      <c r="E46" s="6"/>
-      <c r="G46" s="8" t="str">
+      <c r="B46" s="13"/>
+      <c r="C46" s="12"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="12"/>
+      <c r="G46" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H46" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I46" s="1">
         <f t="shared" si="4"/>
@@ -1885,17 +2545,17 @@
       </c>
     </row>
     <row r="47" spans="2:9">
-      <c r="B47" s="7"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="6"/>
-      <c r="G47" s="8" t="str">
+      <c r="B47" s="13"/>
+      <c r="C47" s="12"/>
+      <c r="D47" s="13"/>
+      <c r="E47" s="12"/>
+      <c r="G47" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H47" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I47" s="1">
         <f t="shared" si="4"/>
@@ -1903,17 +2563,17 @@
       </c>
     </row>
     <row r="48" spans="2:9">
-      <c r="B48" s="7"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="7"/>
-      <c r="E48" s="6"/>
-      <c r="G48" s="8" t="str">
+      <c r="B48" s="13"/>
+      <c r="C48" s="12"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="12"/>
+      <c r="G48" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H48" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I48" s="1">
         <f t="shared" si="4"/>
@@ -1921,17 +2581,17 @@
       </c>
     </row>
     <row r="49" spans="2:9">
-      <c r="B49" s="7"/>
-      <c r="C49" s="6"/>
-      <c r="D49" s="7"/>
-      <c r="E49" s="6"/>
-      <c r="G49" s="8" t="str">
+      <c r="B49" s="13"/>
+      <c r="C49" s="12"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="12"/>
+      <c r="G49" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H49" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I49" s="1">
         <f t="shared" si="4"/>
@@ -1939,17 +2599,17 @@
       </c>
     </row>
     <row r="50" spans="2:9">
-      <c r="B50" s="7"/>
-      <c r="C50" s="6"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="6"/>
-      <c r="G50" s="8" t="str">
+      <c r="B50" s="13"/>
+      <c r="C50" s="12"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="12"/>
+      <c r="G50" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H50" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I50" s="1">
         <f t="shared" si="4"/>
@@ -1957,17 +2617,17 @@
       </c>
     </row>
     <row r="51" spans="2:9">
-      <c r="B51" s="7"/>
-      <c r="C51" s="6"/>
-      <c r="D51" s="7"/>
-      <c r="E51" s="6"/>
-      <c r="G51" s="8" t="str">
+      <c r="B51" s="13"/>
+      <c r="C51" s="12"/>
+      <c r="D51" s="13"/>
+      <c r="E51" s="12"/>
+      <c r="G51" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H51" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I51" s="1">
         <f t="shared" si="4"/>
@@ -1975,17 +2635,17 @@
       </c>
     </row>
     <row r="52" spans="2:9">
-      <c r="B52" s="7"/>
-      <c r="C52" s="6"/>
-      <c r="D52" s="7"/>
-      <c r="E52" s="6"/>
-      <c r="G52" s="8" t="str">
+      <c r="B52" s="13"/>
+      <c r="C52" s="12"/>
+      <c r="D52" s="13"/>
+      <c r="E52" s="12"/>
+      <c r="G52" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H52" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I52" s="1">
         <f t="shared" si="4"/>
@@ -1993,17 +2653,17 @@
       </c>
     </row>
     <row r="53" spans="2:9">
-      <c r="B53" s="7"/>
-      <c r="C53" s="6"/>
-      <c r="D53" s="7"/>
-      <c r="E53" s="6"/>
-      <c r="G53" s="8" t="str">
+      <c r="B53" s="13"/>
+      <c r="C53" s="12"/>
+      <c r="D53" s="13"/>
+      <c r="E53" s="12"/>
+      <c r="G53" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H53" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I53" s="1">
         <f t="shared" si="4"/>
@@ -2011,17 +2671,17 @@
       </c>
     </row>
     <row r="54" spans="2:9">
-      <c r="B54" s="7"/>
-      <c r="C54" s="6"/>
-      <c r="D54" s="7"/>
-      <c r="E54" s="6"/>
-      <c r="G54" s="8" t="str">
+      <c r="B54" s="13"/>
+      <c r="C54" s="12"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="12"/>
+      <c r="G54" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H54" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I54" s="1">
         <f t="shared" si="4"/>
@@ -2029,17 +2689,17 @@
       </c>
     </row>
     <row r="55" spans="2:9">
-      <c r="B55" s="7"/>
-      <c r="C55" s="6"/>
-      <c r="D55" s="7"/>
-      <c r="E55" s="6"/>
-      <c r="G55" s="8" t="str">
+      <c r="B55" s="13"/>
+      <c r="C55" s="12"/>
+      <c r="D55" s="13"/>
+      <c r="E55" s="12"/>
+      <c r="G55" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H55" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I55" s="1">
         <f t="shared" si="4"/>
@@ -2047,17 +2707,17 @@
       </c>
     </row>
     <row r="56" spans="2:9">
-      <c r="B56" s="7"/>
-      <c r="C56" s="6"/>
-      <c r="D56" s="7"/>
-      <c r="E56" s="6"/>
-      <c r="G56" s="8" t="str">
+      <c r="B56" s="13"/>
+      <c r="C56" s="12"/>
+      <c r="D56" s="13"/>
+      <c r="E56" s="12"/>
+      <c r="G56" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H56" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I56" s="1">
         <f t="shared" si="4"/>
@@ -2065,17 +2725,17 @@
       </c>
     </row>
     <row r="57" spans="2:9">
-      <c r="B57" s="7"/>
-      <c r="C57" s="6"/>
-      <c r="D57" s="7"/>
-      <c r="E57" s="6"/>
-      <c r="G57" s="8" t="str">
+      <c r="B57" s="13"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="13"/>
+      <c r="E57" s="12"/>
+      <c r="G57" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H57" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I57" s="1">
         <f t="shared" si="4"/>
@@ -2083,17 +2743,17 @@
       </c>
     </row>
     <row r="58" spans="2:9">
-      <c r="B58" s="7"/>
-      <c r="C58" s="6"/>
-      <c r="D58" s="7"/>
-      <c r="E58" s="6"/>
-      <c r="G58" s="8" t="str">
+      <c r="B58" s="13"/>
+      <c r="C58" s="12"/>
+      <c r="D58" s="13"/>
+      <c r="E58" s="12"/>
+      <c r="G58" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H58" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I58" s="1">
         <f t="shared" si="4"/>
@@ -2101,17 +2761,17 @@
       </c>
     </row>
     <row r="59" spans="2:9">
-      <c r="B59" s="7"/>
-      <c r="C59" s="6"/>
-      <c r="D59" s="7"/>
-      <c r="E59" s="6"/>
-      <c r="G59" s="8" t="str">
+      <c r="B59" s="13"/>
+      <c r="C59" s="12"/>
+      <c r="D59" s="13"/>
+      <c r="E59" s="12"/>
+      <c r="G59" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H59" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I59" s="1">
         <f t="shared" si="4"/>
@@ -2119,14 +2779,14 @@
       </c>
     </row>
     <row r="60" spans="2:9">
-      <c r="B60" s="7"/>
-      <c r="G60" s="8" t="str">
+      <c r="B60" s="13"/>
+      <c r="G60" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H60" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I60" s="1">
         <f t="shared" si="4"/>
@@ -2134,14 +2794,14 @@
       </c>
     </row>
     <row r="61" spans="2:9">
-      <c r="B61" s="7"/>
-      <c r="G61" s="8" t="str">
+      <c r="B61" s="13"/>
+      <c r="G61" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H61" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I61" s="1">
         <f t="shared" si="4"/>
@@ -2149,14 +2809,14 @@
       </c>
     </row>
     <row r="62" spans="2:9">
-      <c r="B62" s="7"/>
-      <c r="G62" s="8" t="str">
+      <c r="B62" s="13"/>
+      <c r="G62" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H62" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I62" s="1">
         <f t="shared" si="4"/>
@@ -2164,14 +2824,14 @@
       </c>
     </row>
     <row r="63" spans="2:9">
-      <c r="B63" s="7"/>
-      <c r="G63" s="8" t="str">
+      <c r="B63" s="13"/>
+      <c r="G63" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H63" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I63" s="1">
         <f t="shared" si="4"/>
@@ -2179,39 +2839,39 @@
       </c>
     </row>
     <row r="64" spans="2:9">
-      <c r="B64" s="7"/>
-      <c r="G64" s="8" t="str">
+      <c r="B64" s="13"/>
+      <c r="G64" s="19" t="str">
         <f t="shared" si="6"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H64" s="1" t="str">
         <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I64" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="15">
-      <c r="A65" s="14" t="s">
+    <row r="65" ht="17.6" spans="1:9">
+      <c r="A65" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B65" s="12" t="s">
+      <c r="B65" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C65" s="13"/>
-      <c r="D65" s="12" t="s">
+      <c r="C65" s="6"/>
+      <c r="D65" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E65" s="13"/>
-      <c r="F65" s="18" t="s">
+      <c r="E65" s="6"/>
+      <c r="F65" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="G65" s="18" t="s">
+      <c r="G65" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="H65" s="18" t="s">
+      <c r="H65" s="21" t="s">
         <v>6</v>
       </c>
       <c r="I65" s="1" t="e">
@@ -2219,218 +2879,218 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="15">
-      <c r="A66" s="15"/>
-      <c r="B66" s="2" t="s">
+    <row r="66" ht="17.6" spans="1:9">
+      <c r="A66" s="7"/>
+      <c r="B66" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C66" s="3" t="s">
+      <c r="C66" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D66" s="2" t="s">
+      <c r="D66" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E66" s="3" t="s">
+      <c r="E66" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F66" s="18"/>
-      <c r="G66" s="18"/>
-      <c r="H66" s="18"/>
+      <c r="F66" s="21"/>
+      <c r="G66" s="21"/>
+      <c r="H66" s="21"/>
       <c r="I66" s="1" t="e">
         <f t="shared" si="4"/>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="67" spans="1:9">
-      <c r="G67" s="8" t="str">
+    <row r="67" spans="7:9">
+      <c r="G67" s="19" t="str">
         <f t="shared" ref="G67:G98" si="8">IF(I67&gt;0,I67,IF(I67=0," ","ERROR"))</f>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H67" s="1" t="str">
         <f>IF(AND(G67&lt;&gt;" ",G67&lt;&gt;"ERROR",H64&lt;&gt;" ",H64&lt;&gt;"ERROR"),G67+H64," ")</f>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I67" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:9">
-      <c r="G68" s="8" t="str">
+    <row r="68" spans="7:9">
+      <c r="G68" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H68" s="1" t="str">
         <f t="shared" ref="H68:H98" si="9">IF(AND(G68&lt;&gt;" ",G68&lt;&gt;"ERROR",H67&lt;&gt;" ",H67&lt;&gt;"ERROR"),G68+H67," ")</f>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I68" s="1">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:9">
-      <c r="G69" s="8" t="str">
+    <row r="69" spans="7:9">
+      <c r="G69" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H69" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I69" s="1">
         <f t="shared" ref="I69:I132" si="10">((D69+E69)-(B69+C69))*24</f>
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:9">
-      <c r="G70" s="8" t="str">
+    <row r="70" spans="7:9">
+      <c r="G70" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H70" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I70" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:9">
-      <c r="G71" s="8" t="str">
+    <row r="71" spans="7:9">
+      <c r="G71" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H71" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I71" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:9">
-      <c r="G72" s="8" t="str">
+    <row r="72" spans="7:9">
+      <c r="G72" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H72" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I72" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:9">
-      <c r="G73" s="8" t="str">
+    <row r="73" spans="7:9">
+      <c r="G73" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H73" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I73" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:9">
-      <c r="G74" s="8" t="str">
+    <row r="74" spans="7:9">
+      <c r="G74" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H74" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I74" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:9">
-      <c r="G75" s="8" t="str">
+    <row r="75" spans="7:9">
+      <c r="G75" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H75" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I75" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:9">
-      <c r="G76" s="8" t="str">
+    <row r="76" spans="7:9">
+      <c r="G76" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H76" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I76" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:9">
-      <c r="G77" s="8" t="str">
+    <row r="77" spans="7:9">
+      <c r="G77" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H77" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I77" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:9">
-      <c r="G78" s="8" t="str">
+    <row r="78" spans="7:9">
+      <c r="G78" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H78" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I78" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:9">
-      <c r="G79" s="8" t="str">
+    <row r="79" spans="7:9">
+      <c r="G79" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H79" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I79" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:9">
-      <c r="G80" s="8" t="str">
+    <row r="80" spans="7:9">
+      <c r="G80" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H80" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I80" s="1">
         <f t="shared" si="10"/>
@@ -2438,13 +3098,13 @@
       </c>
     </row>
     <row r="81" spans="7:9">
-      <c r="G81" s="8" t="str">
+      <c r="G81" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H81" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I81" s="1">
         <f t="shared" si="10"/>
@@ -2452,13 +3112,13 @@
       </c>
     </row>
     <row r="82" spans="7:9">
-      <c r="G82" s="8" t="str">
+      <c r="G82" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H82" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I82" s="1">
         <f t="shared" si="10"/>
@@ -2466,13 +3126,13 @@
       </c>
     </row>
     <row r="83" spans="7:9">
-      <c r="G83" s="8" t="str">
+      <c r="G83" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H83" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I83" s="1">
         <f t="shared" si="10"/>
@@ -2480,13 +3140,13 @@
       </c>
     </row>
     <row r="84" spans="7:9">
-      <c r="G84" s="8" t="str">
+      <c r="G84" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H84" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I84" s="1">
         <f t="shared" si="10"/>
@@ -2494,13 +3154,13 @@
       </c>
     </row>
     <row r="85" spans="7:9">
-      <c r="G85" s="8" t="str">
+      <c r="G85" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H85" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I85" s="1">
         <f t="shared" si="10"/>
@@ -2508,13 +3168,13 @@
       </c>
     </row>
     <row r="86" spans="7:9">
-      <c r="G86" s="8" t="str">
+      <c r="G86" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H86" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I86" s="1">
         <f t="shared" si="10"/>
@@ -2522,13 +3182,13 @@
       </c>
     </row>
     <row r="87" spans="7:9">
-      <c r="G87" s="8" t="str">
+      <c r="G87" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H87" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I87" s="1">
         <f t="shared" si="10"/>
@@ -2536,13 +3196,13 @@
       </c>
     </row>
     <row r="88" spans="7:9">
-      <c r="G88" s="8" t="str">
+      <c r="G88" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H88" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I88" s="1">
         <f t="shared" si="10"/>
@@ -2550,13 +3210,13 @@
       </c>
     </row>
     <row r="89" spans="7:9">
-      <c r="G89" s="8" t="str">
+      <c r="G89" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H89" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I89" s="1">
         <f t="shared" si="10"/>
@@ -2564,13 +3224,13 @@
       </c>
     </row>
     <row r="90" spans="7:9">
-      <c r="G90" s="8" t="str">
+      <c r="G90" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H90" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I90" s="1">
         <f t="shared" si="10"/>
@@ -2578,13 +3238,13 @@
       </c>
     </row>
     <row r="91" spans="7:9">
-      <c r="G91" s="8" t="str">
+      <c r="G91" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H91" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I91" s="1">
         <f t="shared" si="10"/>
@@ -2592,13 +3252,13 @@
       </c>
     </row>
     <row r="92" spans="7:9">
-      <c r="G92" s="8" t="str">
+      <c r="G92" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H92" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I92" s="1">
         <f t="shared" si="10"/>
@@ -2606,13 +3266,13 @@
       </c>
     </row>
     <row r="93" spans="7:9">
-      <c r="G93" s="8" t="str">
+      <c r="G93" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H93" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I93" s="1">
         <f t="shared" si="10"/>
@@ -2620,13 +3280,13 @@
       </c>
     </row>
     <row r="94" spans="7:9">
-      <c r="G94" s="8" t="str">
+      <c r="G94" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H94" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I94" s="1">
         <f t="shared" si="10"/>
@@ -2634,13 +3294,13 @@
       </c>
     </row>
     <row r="95" spans="7:9">
-      <c r="G95" s="8" t="str">
+      <c r="G95" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H95" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I95" s="1">
         <f t="shared" si="10"/>
@@ -2648,66 +3308,66 @@
       </c>
     </row>
     <row r="96" spans="7:9">
-      <c r="G96" s="8" t="str">
+      <c r="G96" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H96" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I96" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:9">
-      <c r="G97" s="8" t="str">
+    <row r="97" spans="7:9">
+      <c r="G97" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H97" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I97" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:9">
-      <c r="G98" s="8" t="str">
+    <row r="98" spans="7:9">
+      <c r="G98" s="19" t="str">
         <f t="shared" si="8"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H98" s="1" t="str">
         <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I98" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="15">
-      <c r="A99" s="14" t="s">
+    <row r="99" ht="17.6" spans="1:9">
+      <c r="A99" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B99" s="12" t="s">
+      <c r="B99" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C99" s="13"/>
-      <c r="D99" s="12" t="s">
+      <c r="C99" s="6"/>
+      <c r="D99" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E99" s="13"/>
-      <c r="F99" s="18" t="s">
+      <c r="E99" s="6"/>
+      <c r="F99" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="G99" s="18" t="s">
+      <c r="G99" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="H99" s="18" t="s">
+      <c r="H99" s="21" t="s">
         <v>6</v>
       </c>
       <c r="I99" s="1" t="e">
@@ -2715,190 +3375,190 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="15">
-      <c r="A100" s="15"/>
-      <c r="B100" s="2" t="s">
+    <row r="100" ht="17.6" spans="1:9">
+      <c r="A100" s="7"/>
+      <c r="B100" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="C100" s="3" t="s">
+      <c r="C100" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D100" s="2" t="s">
+      <c r="D100" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="E100" s="3" t="s">
+      <c r="E100" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="F100" s="18"/>
-      <c r="G100" s="18"/>
-      <c r="H100" s="18"/>
+      <c r="F100" s="21"/>
+      <c r="G100" s="21"/>
+      <c r="H100" s="21"/>
       <c r="I100" s="1" t="e">
         <f t="shared" si="10"/>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="101" spans="1:9">
-      <c r="G101" s="8" t="str">
+    <row r="101" spans="7:9">
+      <c r="G101" s="19" t="str">
         <f t="shared" ref="G101:G132" si="11">IF(I101&gt;0,I101,IF(I101=0," ","ERROR"))</f>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H101" s="1" t="str">
         <f>IF(AND(G101&lt;&gt;" ",G101&lt;&gt;"ERROR",H98&lt;&gt;" ",H98&lt;&gt;"ERROR"),G101+H98," ")</f>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I101" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:9">
-      <c r="G102" s="8" t="str">
+    <row r="102" spans="7:9">
+      <c r="G102" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H102" s="1" t="str">
         <f t="shared" ref="H102:H132" si="12">IF(AND(G102&lt;&gt;" ",G102&lt;&gt;"ERROR",H101&lt;&gt;" ",H101&lt;&gt;"ERROR"),G102+H101," ")</f>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I102" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:9">
-      <c r="G103" s="8" t="str">
+    <row r="103" spans="7:9">
+      <c r="G103" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H103" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I103" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:9">
-      <c r="G104" s="8" t="str">
+    <row r="104" spans="7:9">
+      <c r="G104" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H104" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I104" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:9">
-      <c r="G105" s="8" t="str">
+    <row r="105" spans="7:9">
+      <c r="G105" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H105" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I105" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:9">
-      <c r="G106" s="8" t="str">
+    <row r="106" spans="7:9">
+      <c r="G106" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H106" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I106" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:9">
-      <c r="G107" s="8" t="str">
+    <row r="107" spans="7:9">
+      <c r="G107" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H107" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I107" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:9">
-      <c r="G108" s="8" t="str">
+    <row r="108" spans="7:9">
+      <c r="G108" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H108" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I108" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:9">
-      <c r="G109" s="8" t="str">
+    <row r="109" spans="7:9">
+      <c r="G109" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H109" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I109" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:9">
-      <c r="G110" s="8" t="str">
+    <row r="110" spans="7:9">
+      <c r="G110" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H110" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I110" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:9">
-      <c r="G111" s="8" t="str">
+    <row r="111" spans="7:9">
+      <c r="G111" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H111" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I111" s="1">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:9">
-      <c r="G112" s="8" t="str">
+    <row r="112" spans="7:9">
+      <c r="G112" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H112" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I112" s="1">
         <f t="shared" si="10"/>
@@ -2906,13 +3566,13 @@
       </c>
     </row>
     <row r="113" spans="7:9">
-      <c r="G113" s="8" t="str">
+      <c r="G113" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H113" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I113" s="1">
         <f t="shared" si="10"/>
@@ -2920,13 +3580,13 @@
       </c>
     </row>
     <row r="114" spans="7:9">
-      <c r="G114" s="8" t="str">
+      <c r="G114" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H114" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I114" s="1">
         <f t="shared" si="10"/>
@@ -2934,13 +3594,13 @@
       </c>
     </row>
     <row r="115" spans="7:9">
-      <c r="G115" s="8" t="str">
+      <c r="G115" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H115" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I115" s="1">
         <f t="shared" si="10"/>
@@ -2948,13 +3608,13 @@
       </c>
     </row>
     <row r="116" spans="7:9">
-      <c r="G116" s="8" t="str">
+      <c r="G116" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H116" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I116" s="1">
         <f t="shared" si="10"/>
@@ -2962,13 +3622,13 @@
       </c>
     </row>
     <row r="117" spans="7:9">
-      <c r="G117" s="8" t="str">
+      <c r="G117" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H117" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I117" s="1">
         <f t="shared" si="10"/>
@@ -2976,13 +3636,13 @@
       </c>
     </row>
     <row r="118" spans="7:9">
-      <c r="G118" s="8" t="str">
+      <c r="G118" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H118" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I118" s="1">
         <f t="shared" si="10"/>
@@ -2990,13 +3650,13 @@
       </c>
     </row>
     <row r="119" spans="7:9">
-      <c r="G119" s="8" t="str">
+      <c r="G119" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H119" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I119" s="1">
         <f t="shared" si="10"/>
@@ -3004,13 +3664,13 @@
       </c>
     </row>
     <row r="120" spans="7:9">
-      <c r="G120" s="8" t="str">
+      <c r="G120" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H120" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I120" s="1">
         <f t="shared" si="10"/>
@@ -3018,13 +3678,13 @@
       </c>
     </row>
     <row r="121" spans="7:9">
-      <c r="G121" s="8" t="str">
+      <c r="G121" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H121" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I121" s="1">
         <f t="shared" si="10"/>
@@ -3032,13 +3692,13 @@
       </c>
     </row>
     <row r="122" spans="7:9">
-      <c r="G122" s="8" t="str">
+      <c r="G122" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H122" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I122" s="1">
         <f t="shared" si="10"/>
@@ -3046,13 +3706,13 @@
       </c>
     </row>
     <row r="123" spans="7:9">
-      <c r="G123" s="8" t="str">
+      <c r="G123" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H123" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I123" s="1">
         <f t="shared" si="10"/>
@@ -3060,13 +3720,13 @@
       </c>
     </row>
     <row r="124" spans="7:9">
-      <c r="G124" s="8" t="str">
+      <c r="G124" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H124" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I124" s="1">
         <f t="shared" si="10"/>
@@ -3074,13 +3734,13 @@
       </c>
     </row>
     <row r="125" spans="7:9">
-      <c r="G125" s="8" t="str">
+      <c r="G125" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H125" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I125" s="1">
         <f t="shared" si="10"/>
@@ -3088,13 +3748,13 @@
       </c>
     </row>
     <row r="126" spans="7:9">
-      <c r="G126" s="8" t="str">
+      <c r="G126" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H126" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I126" s="1">
         <f t="shared" si="10"/>
@@ -3102,13 +3762,13 @@
       </c>
     </row>
     <row r="127" spans="7:9">
-      <c r="G127" s="8" t="str">
+      <c r="G127" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H127" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I127" s="1">
         <f t="shared" si="10"/>
@@ -3116,13 +3776,13 @@
       </c>
     </row>
     <row r="128" spans="7:9">
-      <c r="G128" s="8" t="str">
+      <c r="G128" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H128" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I128" s="1">
         <f t="shared" si="10"/>
@@ -3130,13 +3790,13 @@
       </c>
     </row>
     <row r="129" spans="7:9">
-      <c r="G129" s="8" t="str">
+      <c r="G129" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H129" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I129" s="1">
         <f t="shared" si="10"/>
@@ -3144,13 +3804,13 @@
       </c>
     </row>
     <row r="130" spans="7:9">
-      <c r="G130" s="8" t="str">
+      <c r="G130" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H130" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I130" s="1">
         <f t="shared" si="10"/>
@@ -3158,13 +3818,13 @@
       </c>
     </row>
     <row r="131" spans="7:9">
-      <c r="G131" s="8" t="str">
+      <c r="G131" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H131" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I131" s="1">
         <f t="shared" si="10"/>
@@ -3172,13 +3832,13 @@
       </c>
     </row>
     <row r="132" spans="7:9">
-      <c r="G132" s="8" t="str">
+      <c r="G132" s="19" t="str">
         <f t="shared" si="11"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="H132" s="1" t="str">
         <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
+        <v> </v>
       </c>
       <c r="I132" s="1">
         <f t="shared" si="10"/>
@@ -3187,14 +3847,11 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="H65:H66"/>
-    <mergeCell ref="H99:H100"/>
-    <mergeCell ref="F65:F66"/>
-    <mergeCell ref="F99:F100"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="G65:G66"/>
-    <mergeCell ref="G99:G100"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="D31:E31"/>
     <mergeCell ref="B65:C65"/>
     <mergeCell ref="D65:E65"/>
     <mergeCell ref="B99:C99"/>
@@ -3203,26 +3860,30 @@
     <mergeCell ref="A31:A32"/>
     <mergeCell ref="A65:A66"/>
     <mergeCell ref="A99:A100"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="D31:E31"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="F31:F32"/>
+    <mergeCell ref="F65:F66"/>
+    <mergeCell ref="F99:F100"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="G65:G66"/>
+    <mergeCell ref="G99:G100"/>
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="H31:H32"/>
+    <mergeCell ref="H65:H66"/>
+    <mergeCell ref="H99:H100"/>
   </mergeCells>
-  <pageMargins left="0.74803149606299202" right="0.74803149606299202" top="0.98425196850393704" bottom="0.98425196850393704" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.748031496062992" right="0.748031496062992" top="0.984251968503937" bottom="0.984251968503937" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="landscape"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="12.6"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.2"/>
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -3231,9 +3892,10 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="12.6"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.2"/>
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>